<commit_message>
Extend KTB RTD monitoring and decision support
</commit_message>
<xml_diff>
--- a/국채선물 호가창.xlsx
+++ b/국채선물 호가창.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Check\Documents\Codex\2026-10-02\referenced-chatgpt-conversation-this-is-an\outputs\ktb_rtd_monitor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Check\Downloads\금융개발\ktb_rtd_monitor\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14700" windowHeight="11310"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14700" windowHeight="11310" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="추가RTD" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>매수
 잔량</t>
@@ -65,6 +66,46 @@
   </si>
   <si>
     <t>체결가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3선 외국인 누적 매수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">3선 외국인 누적 매도 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3선 선물가격</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10선 외국인 누적 매수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">10선 외국인 누적 매도 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10선 선물가격</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>현물 3년(%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>현물 10년(%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3선 선물수익률 (%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10선 선물수익률 (%)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -72,7 +113,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -94,6 +138,14 @@
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
@@ -173,12 +225,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -197,6 +252,9 @@
     <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -206,11 +264,12 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="쉼표 [0]" xfId="1" builtinId="6"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -231,490 +290,548 @@
   <volType type="realTimeData">
     <main first="checkexpert.rtd">
       <tp>
-        <v>104.81</v>
+        <v>78086</v>
+        <stp/>
+        <stp>17966^11</stp>
+        <stp>*016</stp>
+        <tr r="B8" s="2"/>
+      </tp>
+      <tp>
+        <v>119111</v>
+        <stp/>
+        <stp>17967^11</stp>
+        <stp>*017</stp>
+        <tr r="B3" s="2"/>
+      </tp>
+      <tp>
+        <v>118204</v>
+        <stp/>
+        <stp>17966^11</stp>
+        <stp>*017</stp>
+        <tr r="B4" s="2"/>
+      </tp>
+      <tp>
+        <v>78687</v>
+        <stp/>
+        <stp>17967^11</stp>
+        <stp>*016</stp>
+        <tr r="B7" s="2"/>
+      </tp>
+      <tp>
+        <v>3.8610000000000002</v>
+        <stp/>
+        <stp>15175</stp>
+        <stp>KTBS03*161</stp>
+        <tr r="B1" s="2"/>
+      </tp>
+      <tp>
+        <v>4.1879999999999997</v>
+        <stp/>
+        <stp>15175</stp>
+        <stp>KTBS10*161</stp>
+        <tr r="B2" s="2"/>
+      </tp>
+      <tp>
+        <v>4.2210000000000001</v>
+        <stp/>
+        <stp>15175</stp>
+        <stp>KXFA020</stp>
+        <tr r="B10" s="2"/>
+      </tp>
+      <tp>
+        <v>3.948</v>
+        <stp/>
+        <stp>15175</stp>
+        <stp>KBFA020</stp>
+        <tr r="B6" s="2"/>
+      </tp>
+      <tp>
+        <v>106.3</v>
         <stp/>
         <stp>15001</stp>
         <stp>KXFA020</stp>
+        <tr r="B9" s="2"/>
         <tr r="O2" s="1"/>
       </tp>
       <tp>
-        <v>102.63</v>
+        <v>102.95</v>
         <stp/>
         <stp>15001</stp>
         <stp>KBFA020</stp>
+        <tr r="B5" s="2"/>
         <tr r="G2" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>106.33</v>
         <stp/>
         <stp>14504</stp>
         <stp>KXFA020</stp>
         <tr r="L3" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>106.34</v>
         <stp/>
         <stp>14505</stp>
         <stp>KXFA020</stp>
         <tr r="L2" s="1"/>
       </tp>
       <tp>
-        <v>104.85</v>
+        <v>106.3</v>
         <stp/>
         <stp>14501</stp>
         <stp>KXFA020</stp>
         <tr r="L6" s="1"/>
       </tp>
       <tp>
-        <v>104.86</v>
+        <v>106.31</v>
         <stp/>
         <stp>14502</stp>
         <stp>KXFA020</stp>
         <tr r="L5" s="1"/>
       </tp>
       <tp>
-        <v>104.87</v>
+        <v>106.32</v>
         <stp/>
         <stp>14503</stp>
         <stp>KXFA020</stp>
         <tr r="L4" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>3</v>
         <stp/>
         <stp>14514</stp>
         <stp>KXFA020</stp>
         <tr r="K3" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>27</v>
         <stp/>
         <stp>14515</stp>
         <stp>KXFA020</stp>
         <tr r="K2" s="1"/>
       </tp>
       <tp>
-        <v>230</v>
+        <v>329</v>
         <stp/>
         <stp>14511</stp>
         <stp>KXFA020</stp>
         <tr r="K6" s="1"/>
       </tp>
       <tp>
+        <v>8</v>
+        <stp/>
+        <stp>14512</stp>
+        <stp>KXFA020</stp>
+        <tr r="K5" s="1"/>
+      </tp>
+      <tp>
+        <v>13</v>
+        <stp/>
+        <stp>14513</stp>
+        <stp>KXFA020</stp>
+        <tr r="K4" s="1"/>
+      </tp>
+      <tp>
+        <v>106.26</v>
+        <stp/>
+        <stp>14534</stp>
+        <stp>KXFA020</stp>
+        <tr r="L10" s="1"/>
+      </tp>
+      <tp>
+        <v>106.25</v>
+        <stp/>
+        <stp>14535</stp>
+        <stp>KXFA020</stp>
+        <tr r="L11" s="1"/>
+      </tp>
+      <tp>
+        <v>106.29</v>
+        <stp/>
+        <stp>14531</stp>
+        <stp>KXFA020</stp>
+        <tr r="L7" s="1"/>
+      </tp>
+      <tp>
+        <v>106.28</v>
+        <stp/>
+        <stp>14532</stp>
+        <stp>KXFA020</stp>
+        <tr r="L8" s="1"/>
+      </tp>
+      <tp>
+        <v>106.27</v>
+        <stp/>
+        <stp>14533</stp>
+        <stp>KXFA020</stp>
+        <tr r="L9" s="1"/>
+      </tp>
+      <tp>
+        <v>71</v>
+        <stp/>
+        <stp>14544</stp>
+        <stp>KXFA020</stp>
+        <tr r="M10" s="1"/>
+      </tp>
+      <tp>
+        <v>81</v>
+        <stp/>
+        <stp>14545</stp>
+        <stp>KXFA020</stp>
+        <tr r="M11" s="1"/>
+      </tp>
+      <tp>
+        <v>117</v>
+        <stp/>
+        <stp>14541</stp>
+        <stp>KXFA020</stp>
+        <tr r="M7" s="1"/>
+      </tp>
+      <tp>
+        <v>102</v>
+        <stp/>
+        <stp>14542</stp>
+        <stp>KXFA020</stp>
+        <tr r="M8" s="1"/>
+      </tp>
+      <tp>
+        <v>130</v>
+        <stp/>
+        <stp>14543</stp>
+        <stp>KXFA020</stp>
+        <tr r="M9" s="1"/>
+      </tp>
+      <tp>
+        <v>14</v>
+        <stp/>
+        <stp>14579</stp>
+        <stp>KXFA020</stp>
+        <tr r="J6" s="1"/>
+      </tp>
+      <tp>
+        <v>7</v>
+        <stp/>
+        <stp>14589</stp>
+        <stp>KXFA020</stp>
+        <tr r="N9" s="1"/>
+      </tp>
+      <tp>
+        <v>7</v>
+        <stp/>
+        <stp>14585</stp>
+        <stp>KXFA020</stp>
+        <tr r="N8" s="1"/>
+      </tp>
+      <tp>
+        <v>7</v>
+        <stp/>
+        <stp>14587</stp>
+        <stp>KXFA020</stp>
+        <tr r="J4" s="1"/>
+      </tp>
+      <tp>
+        <v>8</v>
+        <stp/>
+        <stp>14581</stp>
+        <stp>KXFA020</stp>
+        <tr r="N7" s="1"/>
+      </tp>
+      <tp>
+        <v>4</v>
+        <stp/>
+        <stp>14583</stp>
+        <stp>KXFA020</stp>
+        <tr r="J5" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>14595</stp>
+        <stp>KXFA020</stp>
+        <tr r="J2" s="1"/>
+      </tp>
+      <tp>
+        <v>4</v>
+        <stp/>
+        <stp>14597</stp>
+        <stp>KXFA020</stp>
+        <tr r="N11" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>14591</stp>
+        <stp>KXFA020</stp>
+        <tr r="J3" s="1"/>
+      </tp>
+      <tp>
+        <v>4</v>
+        <stp/>
+        <stp>14593</stp>
+        <stp>KXFA020</stp>
+        <tr r="N10" s="1"/>
+      </tp>
+      <tp>
+        <v>18</v>
+        <stp/>
+        <stp>14589</stp>
+        <stp>KBFA020</stp>
+        <tr r="F9" s="1"/>
+      </tp>
+      <tp>
+        <v>23</v>
+        <stp/>
+        <stp>14585</stp>
+        <stp>KBFA020</stp>
+        <tr r="F8" s="1"/>
+      </tp>
+      <tp>
+        <v>8</v>
+        <stp/>
+        <stp>14587</stp>
+        <stp>KBFA020</stp>
+        <tr r="B4" s="1"/>
+      </tp>
+      <tp>
+        <v>19</v>
+        <stp/>
+        <stp>14581</stp>
+        <stp>KBFA020</stp>
+        <tr r="F7" s="1"/>
+      </tp>
+      <tp>
+        <v>5</v>
+        <stp/>
+        <stp>14583</stp>
+        <stp>KBFA020</stp>
+        <tr r="B5" s="1"/>
+      </tp>
+      <tp>
+        <v>20</v>
+        <stp/>
+        <stp>14595</stp>
+        <stp>KBFA020</stp>
+        <tr r="B2" s="1"/>
+      </tp>
+      <tp>
+        <v>16</v>
+        <stp/>
+        <stp>14597</stp>
+        <stp>KBFA020</stp>
+        <tr r="F11" s="1"/>
+      </tp>
+      <tp>
         <v>10</v>
         <stp/>
+        <stp>14591</stp>
+        <stp>KBFA020</stp>
+        <tr r="B3" s="1"/>
+      </tp>
+      <tp>
+        <v>20</v>
+        <stp/>
+        <stp>14593</stp>
+        <stp>KBFA020</stp>
+        <tr r="F10" s="1"/>
+      </tp>
+      <tp>
+        <v>102.92</v>
+        <stp/>
+        <stp>14534</stp>
+        <stp>KBFA020</stp>
+        <tr r="D10" s="1"/>
+      </tp>
+      <tp>
+        <v>102.91</v>
+        <stp/>
+        <stp>14535</stp>
+        <stp>KBFA020</stp>
+        <tr r="D11" s="1"/>
+      </tp>
+      <tp>
+        <v>102.95</v>
+        <stp/>
+        <stp>14531</stp>
+        <stp>KBFA020</stp>
+        <tr r="D7" s="1"/>
+      </tp>
+      <tp>
+        <v>102.94</v>
+        <stp/>
+        <stp>14532</stp>
+        <stp>KBFA020</stp>
+        <tr r="D8" s="1"/>
+      </tp>
+      <tp>
+        <v>102.93</v>
+        <stp/>
+        <stp>14533</stp>
+        <stp>KBFA020</stp>
+        <tr r="D9" s="1"/>
+      </tp>
+      <tp>
+        <v>102.99</v>
+        <stp/>
+        <stp>14504</stp>
+        <stp>KBFA020</stp>
+        <tr r="D3" s="1"/>
+      </tp>
+      <tp>
+        <v>103</v>
+        <stp/>
+        <stp>14505</stp>
+        <stp>KBFA020</stp>
+        <tr r="D2" s="1"/>
+      </tp>
+      <tp>
+        <v>102.96</v>
+        <stp/>
+        <stp>14501</stp>
+        <stp>KBFA020</stp>
+        <tr r="D6" s="1"/>
+      </tp>
+      <tp>
+        <v>102.97</v>
+        <stp/>
+        <stp>14502</stp>
+        <stp>KBFA020</stp>
+        <tr r="D5" s="1"/>
+      </tp>
+      <tp>
+        <v>102.98</v>
+        <stp/>
+        <stp>14503</stp>
+        <stp>KBFA020</stp>
+        <tr r="D4" s="1"/>
+      </tp>
+      <tp>
+        <v>86</v>
+        <stp/>
+        <stp>14514</stp>
+        <stp>KBFA020</stp>
+        <tr r="C3" s="1"/>
+      </tp>
+      <tp>
+        <v>630</v>
+        <stp/>
+        <stp>14515</stp>
+        <stp>KBFA020</stp>
+        <tr r="C2" s="1"/>
+      </tp>
+      <tp>
+        <v>310</v>
+        <stp/>
+        <stp>14511</stp>
+        <stp>KBFA020</stp>
+        <tr r="C6" s="1"/>
+      </tp>
+      <tp>
+        <v>324</v>
+        <stp/>
         <stp>14512</stp>
-        <stp>KXFA020</stp>
-        <tr r="K5" s="1"/>
-      </tp>
-      <tp>
-        <v>18</v>
+        <stp>KBFA020</stp>
+        <tr r="C5" s="1"/>
+      </tp>
+      <tp>
+        <v>834</v>
         <stp/>
         <stp>14513</stp>
-        <stp>KXFA020</stp>
-        <tr r="K4" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14534</stp>
-        <stp>KXFA020</stp>
-        <tr r="L10" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14535</stp>
-        <stp>KXFA020</stp>
-        <tr r="L11" s="1"/>
-      </tp>
-      <tp>
-        <v>104.84</v>
-        <stp/>
-        <stp>14531</stp>
-        <stp>KXFA020</stp>
-        <tr r="L7" s="1"/>
-      </tp>
-      <tp>
-        <v>104.8</v>
-        <stp/>
-        <stp>14532</stp>
-        <stp>KXFA020</stp>
-        <tr r="L8" s="1"/>
-      </tp>
-      <tp>
-        <v>104.78</v>
-        <stp/>
-        <stp>14533</stp>
-        <stp>KXFA020</stp>
-        <tr r="L9" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
+        <stp>KBFA020</stp>
+        <tr r="C4" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>14579</stp>
+        <stp>KBFA020</stp>
+        <tr r="B6" s="1"/>
+      </tp>
+      <tp>
+        <v>329</v>
         <stp/>
         <stp>14544</stp>
-        <stp>KXFA020</stp>
-        <tr r="M10" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
+        <stp>KBFA020</stp>
+        <tr r="E10" s="1"/>
+      </tp>
+      <tp>
+        <v>722</v>
         <stp/>
         <stp>14545</stp>
-        <stp>KXFA020</stp>
-        <tr r="M11" s="1"/>
-      </tp>
-      <tp>
-        <v>4</v>
+        <stp>KBFA020</stp>
+        <tr r="E11" s="1"/>
+      </tp>
+      <tp>
+        <v>1297</v>
         <stp/>
         <stp>14541</stp>
-        <stp>KXFA020</stp>
-        <tr r="M7" s="1"/>
-      </tp>
-      <tp>
-        <v>50</v>
+        <stp>KBFA020</stp>
+        <tr r="E7" s="1"/>
+      </tp>
+      <tp>
+        <v>422</v>
         <stp/>
         <stp>14542</stp>
-        <stp>KXFA020</stp>
-        <tr r="M8" s="1"/>
-      </tp>
-      <tp>
-        <v>50</v>
+        <stp>KBFA020</stp>
+        <tr r="E8" s="1"/>
+      </tp>
+      <tp>
+        <v>632</v>
         <stp/>
         <stp>14543</stp>
-        <stp>KXFA020</stp>
-        <tr r="M9" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14579</stp>
-        <stp>KXFA020</stp>
-        <tr r="J6" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14589</stp>
-        <stp>KXFA020</stp>
-        <tr r="N9" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14585</stp>
-        <stp>KXFA020</stp>
-        <tr r="N8" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14587</stp>
-        <stp>KXFA020</stp>
-        <tr r="J4" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14581</stp>
-        <stp>KXFA020</stp>
-        <tr r="N7" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14583</stp>
-        <stp>KXFA020</stp>
-        <tr r="J5" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14595</stp>
-        <stp>KXFA020</stp>
-        <tr r="J2" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14597</stp>
-        <stp>KXFA020</stp>
-        <tr r="N11" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14591</stp>
-        <stp>KXFA020</stp>
-        <tr r="J3" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14593</stp>
-        <stp>KXFA020</stp>
-        <tr r="N10" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14589</stp>
-        <stp>KBFA020</stp>
-        <tr r="F9" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14585</stp>
-        <stp>KBFA020</stp>
-        <tr r="F8" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14587</stp>
-        <stp>KBFA020</stp>
-        <tr r="B4" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14581</stp>
-        <stp>KBFA020</stp>
-        <tr r="F7" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14583</stp>
-        <stp>KBFA020</stp>
-        <tr r="B5" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14595</stp>
-        <stp>KBFA020</stp>
-        <tr r="B2" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14597</stp>
-        <stp>KBFA020</stp>
-        <tr r="F11" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14591</stp>
-        <stp>KBFA020</stp>
-        <tr r="B3" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14593</stp>
-        <stp>KBFA020</stp>
-        <tr r="F10" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14534</stp>
-        <stp>KBFA020</stp>
-        <tr r="D10" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14535</stp>
-        <stp>KBFA020</stp>
-        <tr r="D11" s="1"/>
-      </tp>
-      <tp>
-        <v>102.63</v>
-        <stp/>
-        <stp>14531</stp>
-        <stp>KBFA020</stp>
-        <tr r="D7" s="1"/>
-      </tp>
-      <tp>
-        <v>102.62</v>
-        <stp/>
-        <stp>14532</stp>
-        <stp>KBFA020</stp>
-        <tr r="D8" s="1"/>
-      </tp>
-      <tp>
-        <v>102.61</v>
-        <stp/>
-        <stp>14533</stp>
-        <stp>KBFA020</stp>
-        <tr r="D9" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14504</stp>
-        <stp>KBFA020</stp>
-        <tr r="D3" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14505</stp>
-        <stp>KBFA020</stp>
-        <tr r="D2" s="1"/>
-      </tp>
-      <tp>
-        <v>102.64</v>
-        <stp/>
-        <stp>14501</stp>
-        <stp>KBFA020</stp>
-        <tr r="D6" s="1"/>
-      </tp>
-      <tp>
-        <v>102.65</v>
-        <stp/>
-        <stp>14502</stp>
-        <stp>KBFA020</stp>
-        <tr r="D5" s="1"/>
-      </tp>
-      <tp>
-        <v>102.66</v>
-        <stp/>
-        <stp>14503</stp>
-        <stp>KBFA020</stp>
-        <tr r="D4" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14514</stp>
-        <stp>KBFA020</stp>
-        <tr r="C3" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14515</stp>
-        <stp>KBFA020</stp>
-        <tr r="C2" s="1"/>
-      </tp>
-      <tp>
-        <v>200</v>
-        <stp/>
-        <stp>14511</stp>
-        <stp>KBFA020</stp>
-        <tr r="C6" s="1"/>
-      </tp>
-      <tp>
-        <v>815</v>
-        <stp/>
-        <stp>14512</stp>
-        <stp>KBFA020</stp>
-        <tr r="C5" s="1"/>
-      </tp>
-      <tp>
-        <v>180</v>
-        <stp/>
-        <stp>14513</stp>
-        <stp>KBFA020</stp>
-        <tr r="C4" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14579</stp>
-        <stp>KBFA020</stp>
-        <tr r="B6" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14544</stp>
-        <stp>KBFA020</stp>
-        <tr r="E10" s="1"/>
-      </tp>
-      <tp>
-        <v>0</v>
-        <stp/>
-        <stp>14545</stp>
-        <stp>KBFA020</stp>
-        <tr r="E11" s="1"/>
-      </tp>
-      <tp>
-        <v>50</v>
-        <stp/>
-        <stp>14541</stp>
-        <stp>KBFA020</stp>
-        <tr r="E7" s="1"/>
-      </tp>
-      <tp>
-        <v>51</v>
-        <stp/>
-        <stp>14542</stp>
-        <stp>KBFA020</stp>
-        <tr r="E8" s="1"/>
-      </tp>
-      <tp>
-        <v>461</v>
-        <stp/>
-        <stp>14543</stp>
         <stp>KBFA020</stp>
         <tr r="E9" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>30</v>
         <stp/>
         <stp>14625</stp>
         <stp>KXFA020</stp>
         <tr r="J12" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>30</v>
         <stp/>
         <stp>14627</stp>
         <stp>KXFA020</stp>
         <tr r="N12" s="1"/>
       </tp>
       <tp>
-        <v>258</v>
+        <v>380</v>
         <stp/>
         <stp>14621</stp>
         <stp>KXFA020</stp>
         <tr r="K12" s="1"/>
       </tp>
       <tp>
-        <v>104</v>
+        <v>501</v>
         <stp/>
         <stp>14623</stp>
         <stp>KXFA020</stp>
         <tr r="M12" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>45</v>
         <stp/>
         <stp>14625</stp>
         <stp>KBFA020</stp>
         <tr r="B12" s="1"/>
       </tp>
       <tp>
-        <v>0</v>
+        <v>96</v>
         <stp/>
         <stp>14627</stp>
         <stp>KBFA020</stp>
         <tr r="F12" s="1"/>
       </tp>
       <tp>
-        <v>1195</v>
+        <v>2184</v>
         <stp/>
         <stp>14621</stp>
         <stp>KBFA020</stp>
         <tr r="C12" s="1"/>
       </tp>
       <tp>
-        <v>562</v>
+        <v>3402</v>
         <stp/>
         <stp>14623</stp>
         <stp>KBFA020</stp>
@@ -992,362 +1109,362 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="I1" s="8" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="I1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1">
         <f>RTD("checkexpert.rtd",,"14595","KBFA020")</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1">
         <f>RTD("checkexpert.rtd",,"14515","KBFA020")</f>
-        <v>0</v>
+        <v>630</v>
       </c>
       <c r="D2" s="2">
         <f>RTD("checkexpert.rtd",,"14505","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="6">
         <f>RTD("checkexpert.rtd",,"15001","KBFA020")</f>
-        <v>102.63</v>
-      </c>
-      <c r="I2" s="6" t="s">
+        <v>102.95</v>
+      </c>
+      <c r="I2" s="7" t="s">
         <v>1</v>
       </c>
       <c r="J2" s="1">
         <f>RTD("checkexpert.rtd",,"14595","KXFA020")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K2" s="1">
         <f>RTD("checkexpert.rtd",,"14515","KXFA020")</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="L2" s="2">
         <f>RTD("checkexpert.rtd",,"14505","KXFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="9" t="s">
+        <v>106.34</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="6">
         <f>RTD("checkexpert.rtd",,"15001","KXFA020")</f>
-        <v>104.81</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
+      <c r="A3" s="8"/>
       <c r="B3" s="1">
         <f>RTD("checkexpert.rtd",,"14591","KBFA020")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1">
         <f>RTD("checkexpert.rtd",,"14514","KBFA020")</f>
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="D3" s="2">
         <f>RTD("checkexpert.rtd",,"14504","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="I3" s="7"/>
+        <v>102.99</v>
+      </c>
+      <c r="I3" s="8"/>
       <c r="J3" s="1">
         <f>RTD("checkexpert.rtd",,"14591","KXFA020")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K3" s="1">
         <f>RTD("checkexpert.rtd",,"14514","KXFA020")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L3" s="2">
         <f>RTD("checkexpert.rtd",,"14504","KXFA020")</f>
-        <v>0</v>
+        <v>106.33</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="1">
         <f>RTD("checkexpert.rtd",,"14587","KBFA020")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1">
         <f>RTD("checkexpert.rtd",,"14513","KBFA020")</f>
-        <v>180</v>
+        <v>834</v>
       </c>
       <c r="D4" s="2">
         <f>RTD("checkexpert.rtd",,"14503","KBFA020")</f>
-        <v>102.66</v>
-      </c>
-      <c r="I4" s="7"/>
+        <v>102.98</v>
+      </c>
+      <c r="I4" s="8"/>
       <c r="J4" s="1">
         <f>RTD("checkexpert.rtd",,"14587","KXFA020")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K4" s="1">
         <f>RTD("checkexpert.rtd",,"14513","KXFA020")</f>
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L4" s="2">
         <f>RTD("checkexpert.rtd",,"14503","KXFA020")</f>
-        <v>104.87</v>
+        <v>106.32</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
+      <c r="A5" s="8"/>
       <c r="B5" s="1">
         <f>RTD("checkexpert.rtd",,"14583","KBFA020")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C5" s="1">
         <f>RTD("checkexpert.rtd",,"14512","KBFA020")</f>
-        <v>815</v>
+        <v>324</v>
       </c>
       <c r="D5" s="2">
         <f>RTD("checkexpert.rtd",,"14502","KBFA020")</f>
-        <v>102.65</v>
-      </c>
-      <c r="I5" s="7"/>
+        <v>102.97</v>
+      </c>
+      <c r="I5" s="8"/>
       <c r="J5" s="1">
         <f>RTD("checkexpert.rtd",,"14583","KXFA020")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K5" s="1">
         <f>RTD("checkexpert.rtd",,"14512","KXFA020")</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L5" s="5">
         <f>RTD("checkexpert.rtd",,"14502","KXFA020")</f>
-        <v>104.86</v>
+        <v>106.31</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+      <c r="A6" s="8"/>
       <c r="B6" s="1">
         <f>RTD("checkexpert.rtd",,"14579","KBFA020")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" s="1">
         <f>RTD("checkexpert.rtd",,"14511","KBFA020")</f>
-        <v>200</v>
+        <v>310</v>
       </c>
       <c r="D6" s="3">
         <f>RTD("checkexpert.rtd",,"14501","KBFA020")</f>
-        <v>102.64</v>
-      </c>
-      <c r="I6" s="7"/>
+        <v>102.96</v>
+      </c>
+      <c r="I6" s="8"/>
       <c r="J6" s="1">
         <f>RTD("checkexpert.rtd",,"14579","KXFA020")</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K6" s="1">
         <f>RTD("checkexpert.rtd",,"14511","KXFA020")</f>
-        <v>230</v>
+        <v>329</v>
       </c>
       <c r="L6" s="2">
         <f>RTD("checkexpert.rtd",,"14501","KXFA020")</f>
-        <v>104.85</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D7" s="4">
         <f>RTD("checkexpert.rtd",,"14531","KBFA020")</f>
-        <v>102.63</v>
+        <v>102.95</v>
       </c>
       <c r="E7" s="1">
         <f>RTD("checkexpert.rtd",,"14541","KBFA020")</f>
-        <v>50</v>
+        <v>1297</v>
       </c>
       <c r="F7" s="1">
         <f>RTD("checkexpert.rtd",,"14581","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>0</v>
       </c>
       <c r="L7" s="4">
         <f>RTD("checkexpert.rtd",,"14531","KXFA020")</f>
-        <v>104.84</v>
+        <v>106.29</v>
       </c>
       <c r="M7" s="1">
         <f>RTD("checkexpert.rtd",,"14541","KXFA020")</f>
-        <v>4</v>
+        <v>117</v>
       </c>
       <c r="N7" s="1">
         <f>RTD("checkexpert.rtd",,"14581","KXFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="O7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="O7" s="7" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D8" s="4">
         <f>RTD("checkexpert.rtd",,"14532","KBFA020")</f>
-        <v>102.62</v>
+        <v>102.94</v>
       </c>
       <c r="E8" s="1">
         <f>RTD("checkexpert.rtd",,"14542","KBFA020")</f>
-        <v>51</v>
+        <v>422</v>
       </c>
       <c r="F8" s="1">
         <f>RTD("checkexpert.rtd",,"14585","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="7"/>
+        <v>23</v>
+      </c>
+      <c r="G8" s="8"/>
       <c r="L8" s="4">
         <f>RTD("checkexpert.rtd",,"14532","KXFA020")</f>
-        <v>104.8</v>
+        <v>106.28</v>
       </c>
       <c r="M8" s="1">
         <f>RTD("checkexpert.rtd",,"14542","KXFA020")</f>
-        <v>50</v>
+        <v>102</v>
       </c>
       <c r="N8" s="1">
         <f>RTD("checkexpert.rtd",,"14585","KXFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="O8" s="7"/>
+        <v>7</v>
+      </c>
+      <c r="O8" s="8"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D9" s="4">
         <f>RTD("checkexpert.rtd",,"14533","KBFA020")</f>
-        <v>102.61</v>
+        <v>102.93</v>
       </c>
       <c r="E9" s="1">
         <f>RTD("checkexpert.rtd",,"14543","KBFA020")</f>
-        <v>461</v>
+        <v>632</v>
       </c>
       <c r="F9" s="1">
         <f>RTD("checkexpert.rtd",,"14589","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="7"/>
+        <v>18</v>
+      </c>
+      <c r="G9" s="8"/>
       <c r="L9" s="4">
         <f>RTD("checkexpert.rtd",,"14533","KXFA020")</f>
-        <v>104.78</v>
+        <v>106.27</v>
       </c>
       <c r="M9" s="1">
         <f>RTD("checkexpert.rtd",,"14543","KXFA020")</f>
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="N9" s="1">
         <f>RTD("checkexpert.rtd",,"14589","KXFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="O9" s="7"/>
+        <v>7</v>
+      </c>
+      <c r="O9" s="8"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D10" s="4">
         <f>RTD("checkexpert.rtd",,"14534","KBFA020")</f>
-        <v>0</v>
+        <v>102.92</v>
       </c>
       <c r="E10" s="1">
         <f>RTD("checkexpert.rtd",,"14544","KBFA020")</f>
-        <v>0</v>
+        <v>329</v>
       </c>
       <c r="F10" s="1">
         <f>RTD("checkexpert.rtd",,"14593","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="7"/>
+        <v>20</v>
+      </c>
+      <c r="G10" s="8"/>
       <c r="L10" s="4">
         <f>RTD("checkexpert.rtd",,"14534","KXFA020")</f>
-        <v>0</v>
+        <v>106.26</v>
       </c>
       <c r="M10" s="1">
         <f>RTD("checkexpert.rtd",,"14544","KXFA020")</f>
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="N10" s="1">
         <f>RTD("checkexpert.rtd",,"14593","KXFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="O10" s="7"/>
+        <v>4</v>
+      </c>
+      <c r="O10" s="8"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D11" s="4">
         <f>RTD("checkexpert.rtd",,"14535","KBFA020")</f>
-        <v>0</v>
+        <v>102.91</v>
       </c>
       <c r="E11" s="1">
         <f>RTD("checkexpert.rtd",,"14545","KBFA020")</f>
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="F11" s="1">
         <f>RTD("checkexpert.rtd",,"14597","KBFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="7"/>
+        <v>16</v>
+      </c>
+      <c r="G11" s="8"/>
       <c r="L11" s="4">
         <f>RTD("checkexpert.rtd",,"14535","KXFA020")</f>
-        <v>0</v>
+        <v>106.25</v>
       </c>
       <c r="M11" s="1">
         <f>RTD("checkexpert.rtd",,"14545","KXFA020")</f>
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="N11" s="1">
         <f>RTD("checkexpert.rtd",,"14597","KXFA020")</f>
-        <v>0</v>
-      </c>
-      <c r="O11" s="7"/>
+        <v>4</v>
+      </c>
+      <c r="O11" s="8"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B12">
         <f>RTD("checkexpert.rtd",,"14625","KBFA020")</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C12">
         <f>RTD("checkexpert.rtd",,"14621","KBFA020")</f>
-        <v>1195</v>
+        <v>2184</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
         <f>RTD("checkexpert.rtd",,"14623","KBFA020")</f>
-        <v>562</v>
+        <v>3402</v>
       </c>
       <c r="F12">
         <f>RTD("checkexpert.rtd",,"14627","KBFA020")</f>
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="J12">
         <f>RTD("checkexpert.rtd",,"14625","KXFA020")</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K12">
         <f>RTD("checkexpert.rtd",,"14621","KXFA020")</f>
-        <v>258</v>
+        <v>380</v>
       </c>
       <c r="M12">
         <f>RTD("checkexpert.rtd",,"14623","KXFA020")</f>
-        <v>104</v>
+        <v>501</v>
       </c>
       <c r="N12">
         <f>RTD("checkexpert.rtd",,"14627","KXFA020")</f>
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -1392,5 +1509,111 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1">
+        <f>RTD("checkexpert.rtd",,"15175","KTBS03*161")</f>
+        <v>3.8610000000000002</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <f>RTD("checkexpert.rtd",,"15175","KTBS10*161")</f>
+        <v>4.1879999999999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="10">
+        <f>RTD("checkexpert.rtd",,"17967^11","*017")</f>
+        <v>119111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="10">
+        <f>RTD("checkexpert.rtd",,"17966^11","*017")</f>
+        <v>118204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <f>RTD("checkexpert.rtd",,"15001","KBFA020")</f>
+        <v>102.95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <f>RTD("checkexpert.rtd",,"15175","KBFA020")</f>
+        <v>3.948</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="10">
+        <f>RTD("checkexpert.rtd",,"17967^11","*016")</f>
+        <v>78687</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="10">
+        <f>RTD("checkexpert.rtd",,"17966^11","*016")</f>
+        <v>78086</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <f>RTD("checkexpert.rtd",,"15001","KXFA020")</f>
+        <v>106.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10">
+        <f>RTD("checkexpert.rtd",,"15175","KXFA020")</f>
+        <v>4.2210000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add cash-curve relative value analytics
</commit_message>
<xml_diff>
--- a/국채선물 호가창.xlsx
+++ b/국채선물 호가창.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>매수
 잔량</t>
@@ -106,6 +106,10 @@
   </si>
   <si>
     <t>10선 선물수익률 (%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>현물 5년(%)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -255,6 +259,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -263,9 +270,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -290,548 +294,555 @@
   <volType type="realTimeData">
     <main first="checkexpert.rtd">
       <tp>
-        <v>78086</v>
+        <v>52663</v>
         <stp/>
         <stp>17966^11</stp>
         <stp>*016</stp>
         <tr r="B8" s="2"/>
       </tp>
       <tp>
-        <v>119111</v>
+        <v>94277</v>
         <stp/>
         <stp>17967^11</stp>
         <stp>*017</stp>
         <tr r="B3" s="2"/>
       </tp>
       <tp>
-        <v>118204</v>
+        <v>90642</v>
         <stp/>
         <stp>17966^11</stp>
         <stp>*017</stp>
         <tr r="B4" s="2"/>
       </tp>
       <tp>
-        <v>78687</v>
+        <v>53035</v>
         <stp/>
         <stp>17967^11</stp>
         <stp>*016</stp>
         <tr r="B7" s="2"/>
       </tp>
       <tp>
-        <v>3.8610000000000002</v>
+        <v>3.8220000000000001</v>
         <stp/>
         <stp>15175</stp>
         <stp>KTBS03*161</stp>
         <tr r="B1" s="2"/>
       </tp>
       <tp>
-        <v>4.1879999999999997</v>
+        <v>3.9649999999999999</v>
+        <stp/>
+        <stp>15175</stp>
+        <stp>KTBS05*161</stp>
+        <tr r="B11" s="2"/>
+      </tp>
+      <tp>
+        <v>4.16</v>
         <stp/>
         <stp>15175</stp>
         <stp>KTBS10*161</stp>
         <tr r="B2" s="2"/>
       </tp>
       <tp>
-        <v>4.2210000000000001</v>
+        <v>4.1669999999999998</v>
         <stp/>
         <stp>15175</stp>
         <stp>KXFA020</stp>
         <tr r="B10" s="2"/>
       </tp>
       <tp>
-        <v>3.948</v>
+        <v>3.8809999999999998</v>
         <stp/>
         <stp>15175</stp>
         <stp>KBFA020</stp>
         <tr r="B6" s="2"/>
       </tp>
       <tp>
-        <v>106.3</v>
+        <v>106.76</v>
         <stp/>
         <stp>15001</stp>
         <stp>KXFA020</stp>
+        <tr r="O2" s="1"/>
         <tr r="B9" s="2"/>
-        <tr r="O2" s="1"/>
-      </tp>
-      <tp>
-        <v>102.95</v>
+      </tp>
+      <tp>
+        <v>103.14</v>
         <stp/>
         <stp>15001</stp>
         <stp>KBFA020</stp>
+        <tr r="G2" s="1"/>
         <tr r="B5" s="2"/>
-        <tr r="G2" s="1"/>
-      </tp>
-      <tp>
-        <v>106.33</v>
+      </tp>
+      <tp>
+        <v>106.79</v>
         <stp/>
         <stp>14504</stp>
         <stp>KXFA020</stp>
         <tr r="L3" s="1"/>
       </tp>
       <tp>
-        <v>106.34</v>
+        <v>106.8</v>
         <stp/>
         <stp>14505</stp>
         <stp>KXFA020</stp>
         <tr r="L2" s="1"/>
       </tp>
       <tp>
-        <v>106.3</v>
+        <v>106.76</v>
         <stp/>
         <stp>14501</stp>
         <stp>KXFA020</stp>
         <tr r="L6" s="1"/>
       </tp>
       <tp>
-        <v>106.31</v>
+        <v>106.77</v>
         <stp/>
         <stp>14502</stp>
         <stp>KXFA020</stp>
         <tr r="L5" s="1"/>
       </tp>
       <tp>
-        <v>106.32</v>
+        <v>106.78</v>
         <stp/>
         <stp>14503</stp>
         <stp>KXFA020</stp>
         <tr r="L4" s="1"/>
       </tp>
       <tp>
+        <v>84</v>
+        <stp/>
+        <stp>14514</stp>
+        <stp>KXFA020</stp>
+        <tr r="K3" s="1"/>
+      </tp>
+      <tp>
+        <v>160</v>
+        <stp/>
+        <stp>14515</stp>
+        <stp>KXFA020</stp>
+        <tr r="K2" s="1"/>
+      </tp>
+      <tp>
+        <v>24</v>
+        <stp/>
+        <stp>14511</stp>
+        <stp>KXFA020</stp>
+        <tr r="K6" s="1"/>
+      </tp>
+      <tp>
+        <v>132</v>
+        <stp/>
+        <stp>14512</stp>
+        <stp>KXFA020</stp>
+        <tr r="K5" s="1"/>
+      </tp>
+      <tp>
+        <v>100</v>
+        <stp/>
+        <stp>14513</stp>
+        <stp>KXFA020</stp>
+        <tr r="K4" s="1"/>
+      </tp>
+      <tp>
+        <v>106.7</v>
+        <stp/>
+        <stp>14534</stp>
+        <stp>KXFA020</stp>
+        <tr r="L10" s="1"/>
+      </tp>
+      <tp>
+        <v>106.69</v>
+        <stp/>
+        <stp>14535</stp>
+        <stp>KXFA020</stp>
+        <tr r="L11" s="1"/>
+      </tp>
+      <tp>
+        <v>106.75</v>
+        <stp/>
+        <stp>14531</stp>
+        <stp>KXFA020</stp>
+        <tr r="L7" s="1"/>
+      </tp>
+      <tp>
+        <v>106.72</v>
+        <stp/>
+        <stp>14532</stp>
+        <stp>KXFA020</stp>
+        <tr r="L8" s="1"/>
+      </tp>
+      <tp>
+        <v>106.71</v>
+        <stp/>
+        <stp>14533</stp>
+        <stp>KXFA020</stp>
+        <tr r="L9" s="1"/>
+      </tp>
+      <tp>
+        <v>175</v>
+        <stp/>
+        <stp>14544</stp>
+        <stp>KXFA020</stp>
+        <tr r="M10" s="1"/>
+      </tp>
+      <tp>
+        <v>44</v>
+        <stp/>
+        <stp>14545</stp>
+        <stp>KXFA020</stp>
+        <tr r="M11" s="1"/>
+      </tp>
+      <tp>
+        <v>200</v>
+        <stp/>
+        <stp>14541</stp>
+        <stp>KXFA020</stp>
+        <tr r="M7" s="1"/>
+      </tp>
+      <tp>
+        <v>45</v>
+        <stp/>
+        <stp>14542</stp>
+        <stp>KXFA020</stp>
+        <tr r="M8" s="1"/>
+      </tp>
+      <tp>
+        <v>10</v>
+        <stp/>
+        <stp>14543</stp>
+        <stp>KXFA020</stp>
+        <tr r="M9" s="1"/>
+      </tp>
+      <tp>
         <v>3</v>
         <stp/>
+        <stp>14579</stp>
+        <stp>KXFA020</stp>
+        <tr r="J6" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>14589</stp>
+        <stp>KXFA020</stp>
+        <tr r="N9" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>14585</stp>
+        <stp>KXFA020</stp>
+        <tr r="N8" s="1"/>
+      </tp>
+      <tp>
+        <v>13</v>
+        <stp/>
+        <stp>14587</stp>
+        <stp>KXFA020</stp>
+        <tr r="J4" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>14581</stp>
+        <stp>KXFA020</stp>
+        <tr r="N7" s="1"/>
+      </tp>
+      <tp>
+        <v>18</v>
+        <stp/>
+        <stp>14583</stp>
+        <stp>KXFA020</stp>
+        <tr r="J5" s="1"/>
+      </tp>
+      <tp>
+        <v>15</v>
+        <stp/>
+        <stp>14595</stp>
+        <stp>KXFA020</stp>
+        <tr r="J2" s="1"/>
+      </tp>
+      <tp>
+        <v>7</v>
+        <stp/>
+        <stp>14597</stp>
+        <stp>KXFA020</stp>
+        <tr r="N11" s="1"/>
+      </tp>
+      <tp>
+        <v>12</v>
+        <stp/>
+        <stp>14591</stp>
+        <stp>KXFA020</stp>
+        <tr r="J3" s="1"/>
+      </tp>
+      <tp>
+        <v>10</v>
+        <stp/>
+        <stp>14593</stp>
+        <stp>KXFA020</stp>
+        <tr r="N10" s="1"/>
+      </tp>
+      <tp>
+        <v>11</v>
+        <stp/>
+        <stp>14589</stp>
+        <stp>KBFA020</stp>
+        <tr r="F9" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>14585</stp>
+        <stp>KBFA020</stp>
+        <tr r="F8" s="1"/>
+      </tp>
+      <tp>
+        <v>19</v>
+        <stp/>
+        <stp>14587</stp>
+        <stp>KBFA020</stp>
+        <tr r="B4" s="1"/>
+      </tp>
+      <tp>
+        <v>5</v>
+        <stp/>
+        <stp>14581</stp>
+        <stp>KBFA020</stp>
+        <tr r="F7" s="1"/>
+      </tp>
+      <tp>
+        <v>22</v>
+        <stp/>
+        <stp>14583</stp>
+        <stp>KBFA020</stp>
+        <tr r="B5" s="1"/>
+      </tp>
+      <tp>
+        <v>10</v>
+        <stp/>
+        <stp>14595</stp>
+        <stp>KBFA020</stp>
+        <tr r="B2" s="1"/>
+      </tp>
+      <tp>
+        <v>13</v>
+        <stp/>
+        <stp>14597</stp>
+        <stp>KBFA020</stp>
+        <tr r="F11" s="1"/>
+      </tp>
+      <tp>
+        <v>14</v>
+        <stp/>
+        <stp>14591</stp>
+        <stp>KBFA020</stp>
+        <tr r="B3" s="1"/>
+      </tp>
+      <tp>
+        <v>14</v>
+        <stp/>
+        <stp>14593</stp>
+        <stp>KBFA020</stp>
+        <tr r="F10" s="1"/>
+      </tp>
+      <tp>
+        <v>103.1</v>
+        <stp/>
+        <stp>14534</stp>
+        <stp>KBFA020</stp>
+        <tr r="D10" s="1"/>
+      </tp>
+      <tp>
+        <v>103.09</v>
+        <stp/>
+        <stp>14535</stp>
+        <stp>KBFA020</stp>
+        <tr r="D11" s="1"/>
+      </tp>
+      <tp>
+        <v>103.13</v>
+        <stp/>
+        <stp>14531</stp>
+        <stp>KBFA020</stp>
+        <tr r="D7" s="1"/>
+      </tp>
+      <tp>
+        <v>103.12</v>
+        <stp/>
+        <stp>14532</stp>
+        <stp>KBFA020</stp>
+        <tr r="D8" s="1"/>
+      </tp>
+      <tp>
+        <v>103.11</v>
+        <stp/>
+        <stp>14533</stp>
+        <stp>KBFA020</stp>
+        <tr r="D9" s="1"/>
+      </tp>
+      <tp>
+        <v>103.17</v>
+        <stp/>
+        <stp>14504</stp>
+        <stp>KBFA020</stp>
+        <tr r="D3" s="1"/>
+      </tp>
+      <tp>
+        <v>103.18</v>
+        <stp/>
+        <stp>14505</stp>
+        <stp>KBFA020</stp>
+        <tr r="D2" s="1"/>
+      </tp>
+      <tp>
+        <v>103.14</v>
+        <stp/>
+        <stp>14501</stp>
+        <stp>KBFA020</stp>
+        <tr r="D6" s="1"/>
+      </tp>
+      <tp>
+        <v>103.15</v>
+        <stp/>
+        <stp>14502</stp>
+        <stp>KBFA020</stp>
+        <tr r="D5" s="1"/>
+      </tp>
+      <tp>
+        <v>103.16</v>
+        <stp/>
+        <stp>14503</stp>
+        <stp>KBFA020</stp>
+        <tr r="D4" s="1"/>
+      </tp>
+      <tp>
+        <v>298</v>
+        <stp/>
         <stp>14514</stp>
-        <stp>KXFA020</stp>
-        <tr r="K3" s="1"/>
-      </tp>
-      <tp>
-        <v>27</v>
+        <stp>KBFA020</stp>
+        <tr r="C3" s="1"/>
+      </tp>
+      <tp>
+        <v>171</v>
         <stp/>
         <stp>14515</stp>
-        <stp>KXFA020</stp>
-        <tr r="K2" s="1"/>
-      </tp>
-      <tp>
-        <v>329</v>
+        <stp>KBFA020</stp>
+        <tr r="C2" s="1"/>
+      </tp>
+      <tp>
+        <v>370</v>
         <stp/>
         <stp>14511</stp>
-        <stp>KXFA020</stp>
-        <tr r="K6" s="1"/>
-      </tp>
-      <tp>
-        <v>8</v>
+        <stp>KBFA020</stp>
+        <tr r="C6" s="1"/>
+      </tp>
+      <tp>
+        <v>573</v>
         <stp/>
         <stp>14512</stp>
-        <stp>KXFA020</stp>
-        <tr r="K5" s="1"/>
-      </tp>
-      <tp>
-        <v>13</v>
+        <stp>KBFA020</stp>
+        <tr r="C5" s="1"/>
+      </tp>
+      <tp>
+        <v>293</v>
         <stp/>
         <stp>14513</stp>
-        <stp>KXFA020</stp>
-        <tr r="K4" s="1"/>
-      </tp>
-      <tp>
-        <v>106.26</v>
-        <stp/>
-        <stp>14534</stp>
-        <stp>KXFA020</stp>
-        <tr r="L10" s="1"/>
-      </tp>
-      <tp>
-        <v>106.25</v>
-        <stp/>
-        <stp>14535</stp>
-        <stp>KXFA020</stp>
-        <tr r="L11" s="1"/>
-      </tp>
-      <tp>
-        <v>106.29</v>
-        <stp/>
-        <stp>14531</stp>
-        <stp>KXFA020</stp>
-        <tr r="L7" s="1"/>
-      </tp>
-      <tp>
-        <v>106.28</v>
-        <stp/>
-        <stp>14532</stp>
-        <stp>KXFA020</stp>
-        <tr r="L8" s="1"/>
-      </tp>
-      <tp>
-        <v>106.27</v>
-        <stp/>
-        <stp>14533</stp>
-        <stp>KXFA020</stp>
-        <tr r="L9" s="1"/>
+        <stp>KBFA020</stp>
+        <tr r="C4" s="1"/>
+      </tp>
+      <tp>
+        <v>6</v>
+        <stp/>
+        <stp>14579</stp>
+        <stp>KBFA020</stp>
+        <tr r="B6" s="1"/>
+      </tp>
+      <tp>
+        <v>390</v>
+        <stp/>
+        <stp>14544</stp>
+        <stp>KBFA020</stp>
+        <tr r="E10" s="1"/>
+      </tp>
+      <tp>
+        <v>473</v>
+        <stp/>
+        <stp>14545</stp>
+        <stp>KBFA020</stp>
+        <tr r="E11" s="1"/>
+      </tp>
+      <tp>
+        <v>616</v>
+        <stp/>
+        <stp>14541</stp>
+        <stp>KBFA020</stp>
+        <tr r="E7" s="1"/>
+      </tp>
+      <tp>
+        <v>100</v>
+        <stp/>
+        <stp>14542</stp>
+        <stp>KBFA020</stp>
+        <tr r="E8" s="1"/>
+      </tp>
+      <tp>
+        <v>483</v>
+        <stp/>
+        <stp>14543</stp>
+        <stp>KBFA020</stp>
+        <tr r="E9" s="1"/>
+      </tp>
+      <tp>
+        <v>61</v>
+        <stp/>
+        <stp>14625</stp>
+        <stp>KXFA020</stp>
+        <tr r="J12" s="1"/>
+      </tp>
+      <tp>
+        <v>21</v>
+        <stp/>
+        <stp>14627</stp>
+        <stp>KXFA020</stp>
+        <tr r="N12" s="1"/>
+      </tp>
+      <tp>
+        <v>500</v>
+        <stp/>
+        <stp>14621</stp>
+        <stp>KXFA020</stp>
+        <tr r="K12" s="1"/>
+      </tp>
+      <tp>
+        <v>474</v>
+        <stp/>
+        <stp>14623</stp>
+        <stp>KXFA020</stp>
+        <tr r="M12" s="1"/>
       </tp>
       <tp>
         <v>71</v>
         <stp/>
-        <stp>14544</stp>
-        <stp>KXFA020</stp>
-        <tr r="M10" s="1"/>
-      </tp>
-      <tp>
-        <v>81</v>
-        <stp/>
-        <stp>14545</stp>
-        <stp>KXFA020</stp>
-        <tr r="M11" s="1"/>
-      </tp>
-      <tp>
-        <v>117</v>
-        <stp/>
-        <stp>14541</stp>
-        <stp>KXFA020</stp>
-        <tr r="M7" s="1"/>
-      </tp>
-      <tp>
-        <v>102</v>
-        <stp/>
-        <stp>14542</stp>
-        <stp>KXFA020</stp>
-        <tr r="M8" s="1"/>
-      </tp>
-      <tp>
-        <v>130</v>
-        <stp/>
-        <stp>14543</stp>
-        <stp>KXFA020</stp>
-        <tr r="M9" s="1"/>
-      </tp>
-      <tp>
-        <v>14</v>
-        <stp/>
-        <stp>14579</stp>
-        <stp>KXFA020</stp>
-        <tr r="J6" s="1"/>
-      </tp>
-      <tp>
-        <v>7</v>
-        <stp/>
-        <stp>14589</stp>
-        <stp>KXFA020</stp>
-        <tr r="N9" s="1"/>
-      </tp>
-      <tp>
-        <v>7</v>
-        <stp/>
-        <stp>14585</stp>
-        <stp>KXFA020</stp>
-        <tr r="N8" s="1"/>
-      </tp>
-      <tp>
-        <v>7</v>
-        <stp/>
-        <stp>14587</stp>
-        <stp>KXFA020</stp>
-        <tr r="J4" s="1"/>
-      </tp>
-      <tp>
-        <v>8</v>
-        <stp/>
-        <stp>14581</stp>
-        <stp>KXFA020</stp>
-        <tr r="N7" s="1"/>
-      </tp>
-      <tp>
-        <v>4</v>
-        <stp/>
-        <stp>14583</stp>
-        <stp>KXFA020</stp>
-        <tr r="J5" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>14595</stp>
-        <stp>KXFA020</stp>
-        <tr r="J2" s="1"/>
-      </tp>
-      <tp>
-        <v>4</v>
-        <stp/>
-        <stp>14597</stp>
-        <stp>KXFA020</stp>
-        <tr r="N11" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>14591</stp>
-        <stp>KXFA020</stp>
-        <tr r="J3" s="1"/>
-      </tp>
-      <tp>
-        <v>4</v>
-        <stp/>
-        <stp>14593</stp>
-        <stp>KXFA020</stp>
-        <tr r="N10" s="1"/>
-      </tp>
-      <tp>
-        <v>18</v>
-        <stp/>
-        <stp>14589</stp>
-        <stp>KBFA020</stp>
-        <tr r="F9" s="1"/>
-      </tp>
-      <tp>
-        <v>23</v>
-        <stp/>
-        <stp>14585</stp>
-        <stp>KBFA020</stp>
-        <tr r="F8" s="1"/>
-      </tp>
-      <tp>
-        <v>8</v>
-        <stp/>
-        <stp>14587</stp>
-        <stp>KBFA020</stp>
-        <tr r="B4" s="1"/>
-      </tp>
-      <tp>
-        <v>19</v>
-        <stp/>
-        <stp>14581</stp>
-        <stp>KBFA020</stp>
-        <tr r="F7" s="1"/>
-      </tp>
-      <tp>
-        <v>5</v>
-        <stp/>
-        <stp>14583</stp>
-        <stp>KBFA020</stp>
-        <tr r="B5" s="1"/>
-      </tp>
-      <tp>
-        <v>20</v>
-        <stp/>
-        <stp>14595</stp>
-        <stp>KBFA020</stp>
-        <tr r="B2" s="1"/>
-      </tp>
-      <tp>
-        <v>16</v>
-        <stp/>
-        <stp>14597</stp>
-        <stp>KBFA020</stp>
-        <tr r="F11" s="1"/>
-      </tp>
-      <tp>
-        <v>10</v>
-        <stp/>
-        <stp>14591</stp>
-        <stp>KBFA020</stp>
-        <tr r="B3" s="1"/>
-      </tp>
-      <tp>
-        <v>20</v>
-        <stp/>
-        <stp>14593</stp>
-        <stp>KBFA020</stp>
-        <tr r="F10" s="1"/>
-      </tp>
-      <tp>
-        <v>102.92</v>
-        <stp/>
-        <stp>14534</stp>
-        <stp>KBFA020</stp>
-        <tr r="D10" s="1"/>
-      </tp>
-      <tp>
-        <v>102.91</v>
-        <stp/>
-        <stp>14535</stp>
-        <stp>KBFA020</stp>
-        <tr r="D11" s="1"/>
-      </tp>
-      <tp>
-        <v>102.95</v>
-        <stp/>
-        <stp>14531</stp>
-        <stp>KBFA020</stp>
-        <tr r="D7" s="1"/>
-      </tp>
-      <tp>
-        <v>102.94</v>
-        <stp/>
-        <stp>14532</stp>
-        <stp>KBFA020</stp>
-        <tr r="D8" s="1"/>
-      </tp>
-      <tp>
-        <v>102.93</v>
-        <stp/>
-        <stp>14533</stp>
-        <stp>KBFA020</stp>
-        <tr r="D9" s="1"/>
-      </tp>
-      <tp>
-        <v>102.99</v>
-        <stp/>
-        <stp>14504</stp>
-        <stp>KBFA020</stp>
-        <tr r="D3" s="1"/>
-      </tp>
-      <tp>
-        <v>103</v>
-        <stp/>
-        <stp>14505</stp>
-        <stp>KBFA020</stp>
-        <tr r="D2" s="1"/>
-      </tp>
-      <tp>
-        <v>102.96</v>
-        <stp/>
-        <stp>14501</stp>
-        <stp>KBFA020</stp>
-        <tr r="D6" s="1"/>
-      </tp>
-      <tp>
-        <v>102.97</v>
-        <stp/>
-        <stp>14502</stp>
-        <stp>KBFA020</stp>
-        <tr r="D5" s="1"/>
-      </tp>
-      <tp>
-        <v>102.98</v>
-        <stp/>
-        <stp>14503</stp>
-        <stp>KBFA020</stp>
-        <tr r="D4" s="1"/>
-      </tp>
-      <tp>
-        <v>86</v>
-        <stp/>
-        <stp>14514</stp>
-        <stp>KBFA020</stp>
-        <tr r="C3" s="1"/>
-      </tp>
-      <tp>
-        <v>630</v>
-        <stp/>
-        <stp>14515</stp>
-        <stp>KBFA020</stp>
-        <tr r="C2" s="1"/>
-      </tp>
-      <tp>
-        <v>310</v>
-        <stp/>
-        <stp>14511</stp>
-        <stp>KBFA020</stp>
-        <tr r="C6" s="1"/>
-      </tp>
-      <tp>
-        <v>324</v>
-        <stp/>
-        <stp>14512</stp>
-        <stp>KBFA020</stp>
-        <tr r="C5" s="1"/>
-      </tp>
-      <tp>
-        <v>834</v>
-        <stp/>
-        <stp>14513</stp>
-        <stp>KBFA020</stp>
-        <tr r="C4" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>14579</stp>
-        <stp>KBFA020</stp>
-        <tr r="B6" s="1"/>
-      </tp>
-      <tp>
-        <v>329</v>
-        <stp/>
-        <stp>14544</stp>
-        <stp>KBFA020</stp>
-        <tr r="E10" s="1"/>
-      </tp>
-      <tp>
-        <v>722</v>
-        <stp/>
-        <stp>14545</stp>
-        <stp>KBFA020</stp>
-        <tr r="E11" s="1"/>
-      </tp>
-      <tp>
-        <v>1297</v>
-        <stp/>
-        <stp>14541</stp>
-        <stp>KBFA020</stp>
-        <tr r="E7" s="1"/>
-      </tp>
-      <tp>
-        <v>422</v>
-        <stp/>
-        <stp>14542</stp>
-        <stp>KBFA020</stp>
-        <tr r="E8" s="1"/>
-      </tp>
-      <tp>
-        <v>632</v>
-        <stp/>
-        <stp>14543</stp>
-        <stp>KBFA020</stp>
-        <tr r="E9" s="1"/>
-      </tp>
-      <tp>
-        <v>30</v>
-        <stp/>
         <stp>14625</stp>
-        <stp>KXFA020</stp>
-        <tr r="J12" s="1"/>
-      </tp>
-      <tp>
-        <v>30</v>
+        <stp>KBFA020</stp>
+        <tr r="B12" s="1"/>
+      </tp>
+      <tp>
+        <v>45</v>
         <stp/>
         <stp>14627</stp>
-        <stp>KXFA020</stp>
-        <tr r="N12" s="1"/>
-      </tp>
-      <tp>
-        <v>380</v>
+        <stp>KBFA020</stp>
+        <tr r="F12" s="1"/>
+      </tp>
+      <tp>
+        <v>1705</v>
         <stp/>
         <stp>14621</stp>
-        <stp>KXFA020</stp>
-        <tr r="K12" s="1"/>
-      </tp>
-      <tp>
-        <v>501</v>
-        <stp/>
-        <stp>14623</stp>
-        <stp>KXFA020</stp>
-        <tr r="M12" s="1"/>
-      </tp>
-      <tp>
-        <v>45</v>
-        <stp/>
-        <stp>14625</stp>
-        <stp>KBFA020</stp>
-        <tr r="B12" s="1"/>
-      </tp>
-      <tp>
-        <v>96</v>
-        <stp/>
-        <stp>14627</stp>
-        <stp>KBFA020</stp>
-        <tr r="F12" s="1"/>
-      </tp>
-      <tp>
-        <v>2184</v>
-        <stp/>
-        <stp>14621</stp>
         <stp>KBFA020</stp>
         <tr r="C12" s="1"/>
       </tp>
       <tp>
-        <v>3402</v>
+        <v>2062</v>
         <stp/>
         <stp>14623</stp>
         <stp>KBFA020</stp>
@@ -1109,362 +1120,362 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="I1" s="9" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="I1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1">
         <f>RTD("checkexpert.rtd",,"14595","KBFA020")</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
         <f>RTD("checkexpert.rtd",,"14515","KBFA020")</f>
-        <v>630</v>
+        <v>171</v>
       </c>
       <c r="D2" s="2">
         <f>RTD("checkexpert.rtd",,"14505","KBFA020")</f>
-        <v>103</v>
+        <v>103.18</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="6">
         <f>RTD("checkexpert.rtd",,"15001","KBFA020")</f>
-        <v>102.95</v>
-      </c>
-      <c r="I2" s="7" t="s">
+        <v>103.14</v>
+      </c>
+      <c r="I2" s="8" t="s">
         <v>1</v>
       </c>
       <c r="J2" s="1">
         <f>RTD("checkexpert.rtd",,"14595","KXFA020")</f>
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="K2" s="1">
         <f>RTD("checkexpert.rtd",,"14515","KXFA020")</f>
-        <v>27</v>
+        <v>160</v>
       </c>
       <c r="L2" s="2">
         <f>RTD("checkexpert.rtd",,"14505","KXFA020")</f>
-        <v>106.34</v>
+        <v>106.8</v>
       </c>
       <c r="N2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="O2" s="6">
         <f>RTD("checkexpert.rtd",,"15001","KXFA020")</f>
-        <v>106.3</v>
+        <v>106.76</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="1">
         <f>RTD("checkexpert.rtd",,"14591","KBFA020")</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1">
         <f>RTD("checkexpert.rtd",,"14514","KBFA020")</f>
-        <v>86</v>
+        <v>298</v>
       </c>
       <c r="D3" s="2">
         <f>RTD("checkexpert.rtd",,"14504","KBFA020")</f>
-        <v>102.99</v>
-      </c>
-      <c r="I3" s="8"/>
+        <v>103.17</v>
+      </c>
+      <c r="I3" s="9"/>
       <c r="J3" s="1">
         <f>RTD("checkexpert.rtd",,"14591","KXFA020")</f>
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K3" s="1">
         <f>RTD("checkexpert.rtd",,"14514","KXFA020")</f>
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="L3" s="2">
         <f>RTD("checkexpert.rtd",,"14504","KXFA020")</f>
-        <v>106.33</v>
+        <v>106.79</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="1">
         <f>RTD("checkexpert.rtd",,"14587","KBFA020")</f>
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C4" s="1">
         <f>RTD("checkexpert.rtd",,"14513","KBFA020")</f>
-        <v>834</v>
+        <v>293</v>
       </c>
       <c r="D4" s="2">
         <f>RTD("checkexpert.rtd",,"14503","KBFA020")</f>
-        <v>102.98</v>
-      </c>
-      <c r="I4" s="8"/>
+        <v>103.16</v>
+      </c>
+      <c r="I4" s="9"/>
       <c r="J4" s="1">
         <f>RTD("checkexpert.rtd",,"14587","KXFA020")</f>
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="K4" s="1">
         <f>RTD("checkexpert.rtd",,"14513","KXFA020")</f>
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="L4" s="2">
         <f>RTD("checkexpert.rtd",,"14503","KXFA020")</f>
-        <v>106.32</v>
+        <v>106.78</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
+      <c r="A5" s="9"/>
       <c r="B5" s="1">
         <f>RTD("checkexpert.rtd",,"14583","KBFA020")</f>
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1">
         <f>RTD("checkexpert.rtd",,"14512","KBFA020")</f>
-        <v>324</v>
+        <v>573</v>
       </c>
       <c r="D5" s="2">
         <f>RTD("checkexpert.rtd",,"14502","KBFA020")</f>
-        <v>102.97</v>
-      </c>
-      <c r="I5" s="8"/>
+        <v>103.15</v>
+      </c>
+      <c r="I5" s="9"/>
       <c r="J5" s="1">
         <f>RTD("checkexpert.rtd",,"14583","KXFA020")</f>
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="K5" s="1">
         <f>RTD("checkexpert.rtd",,"14512","KXFA020")</f>
-        <v>8</v>
+        <v>132</v>
       </c>
       <c r="L5" s="5">
         <f>RTD("checkexpert.rtd",,"14502","KXFA020")</f>
-        <v>106.31</v>
+        <v>106.77</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
+      <c r="A6" s="9"/>
       <c r="B6" s="1">
         <f>RTD("checkexpert.rtd",,"14579","KBFA020")</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C6" s="1">
         <f>RTD("checkexpert.rtd",,"14511","KBFA020")</f>
-        <v>310</v>
+        <v>370</v>
       </c>
       <c r="D6" s="3">
         <f>RTD("checkexpert.rtd",,"14501","KBFA020")</f>
-        <v>102.96</v>
-      </c>
-      <c r="I6" s="8"/>
+        <v>103.14</v>
+      </c>
+      <c r="I6" s="9"/>
       <c r="J6" s="1">
         <f>RTD("checkexpert.rtd",,"14579","KXFA020")</f>
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="K6" s="1">
         <f>RTD("checkexpert.rtd",,"14511","KXFA020")</f>
-        <v>329</v>
+        <v>24</v>
       </c>
       <c r="L6" s="2">
         <f>RTD("checkexpert.rtd",,"14501","KXFA020")</f>
-        <v>106.3</v>
+        <v>106.76</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D7" s="4">
         <f>RTD("checkexpert.rtd",,"14531","KBFA020")</f>
-        <v>102.95</v>
+        <v>103.13</v>
       </c>
       <c r="E7" s="1">
         <f>RTD("checkexpert.rtd",,"14541","KBFA020")</f>
-        <v>1297</v>
+        <v>616</v>
       </c>
       <c r="F7" s="1">
         <f>RTD("checkexpert.rtd",,"14581","KBFA020")</f>
-        <v>19</v>
-      </c>
-      <c r="G7" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>0</v>
       </c>
       <c r="L7" s="4">
         <f>RTD("checkexpert.rtd",,"14531","KXFA020")</f>
-        <v>106.29</v>
+        <v>106.75</v>
       </c>
       <c r="M7" s="1">
         <f>RTD("checkexpert.rtd",,"14541","KXFA020")</f>
-        <v>117</v>
+        <v>200</v>
       </c>
       <c r="N7" s="1">
         <f>RTD("checkexpert.rtd",,"14581","KXFA020")</f>
-        <v>8</v>
-      </c>
-      <c r="O7" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="O7" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D8" s="4">
         <f>RTD("checkexpert.rtd",,"14532","KBFA020")</f>
-        <v>102.94</v>
+        <v>103.12</v>
       </c>
       <c r="E8" s="1">
         <f>RTD("checkexpert.rtd",,"14542","KBFA020")</f>
-        <v>422</v>
+        <v>100</v>
       </c>
       <c r="F8" s="1">
         <f>RTD("checkexpert.rtd",,"14585","KBFA020")</f>
-        <v>23</v>
-      </c>
-      <c r="G8" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="G8" s="9"/>
       <c r="L8" s="4">
         <f>RTD("checkexpert.rtd",,"14532","KXFA020")</f>
-        <v>106.28</v>
+        <v>106.72</v>
       </c>
       <c r="M8" s="1">
         <f>RTD("checkexpert.rtd",,"14542","KXFA020")</f>
-        <v>102</v>
+        <v>45</v>
       </c>
       <c r="N8" s="1">
         <f>RTD("checkexpert.rtd",,"14585","KXFA020")</f>
-        <v>7</v>
-      </c>
-      <c r="O8" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="O8" s="9"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D9" s="4">
         <f>RTD("checkexpert.rtd",,"14533","KBFA020")</f>
-        <v>102.93</v>
+        <v>103.11</v>
       </c>
       <c r="E9" s="1">
         <f>RTD("checkexpert.rtd",,"14543","KBFA020")</f>
-        <v>632</v>
+        <v>483</v>
       </c>
       <c r="F9" s="1">
         <f>RTD("checkexpert.rtd",,"14589","KBFA020")</f>
-        <v>18</v>
-      </c>
-      <c r="G9" s="8"/>
+        <v>11</v>
+      </c>
+      <c r="G9" s="9"/>
       <c r="L9" s="4">
         <f>RTD("checkexpert.rtd",,"14533","KXFA020")</f>
-        <v>106.27</v>
+        <v>106.71</v>
       </c>
       <c r="M9" s="1">
         <f>RTD("checkexpert.rtd",,"14543","KXFA020")</f>
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="N9" s="1">
         <f>RTD("checkexpert.rtd",,"14589","KXFA020")</f>
-        <v>7</v>
-      </c>
-      <c r="O9" s="8"/>
+        <v>1</v>
+      </c>
+      <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D10" s="4">
         <f>RTD("checkexpert.rtd",,"14534","KBFA020")</f>
-        <v>102.92</v>
+        <v>103.1</v>
       </c>
       <c r="E10" s="1">
         <f>RTD("checkexpert.rtd",,"14544","KBFA020")</f>
-        <v>329</v>
+        <v>390</v>
       </c>
       <c r="F10" s="1">
         <f>RTD("checkexpert.rtd",,"14593","KBFA020")</f>
-        <v>20</v>
-      </c>
-      <c r="G10" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="G10" s="9"/>
       <c r="L10" s="4">
         <f>RTD("checkexpert.rtd",,"14534","KXFA020")</f>
-        <v>106.26</v>
+        <v>106.7</v>
       </c>
       <c r="M10" s="1">
         <f>RTD("checkexpert.rtd",,"14544","KXFA020")</f>
-        <v>71</v>
+        <v>175</v>
       </c>
       <c r="N10" s="1">
         <f>RTD("checkexpert.rtd",,"14593","KXFA020")</f>
-        <v>4</v>
-      </c>
-      <c r="O10" s="8"/>
+        <v>10</v>
+      </c>
+      <c r="O10" s="9"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D11" s="4">
         <f>RTD("checkexpert.rtd",,"14535","KBFA020")</f>
-        <v>102.91</v>
+        <v>103.09</v>
       </c>
       <c r="E11" s="1">
         <f>RTD("checkexpert.rtd",,"14545","KBFA020")</f>
-        <v>722</v>
+        <v>473</v>
       </c>
       <c r="F11" s="1">
         <f>RTD("checkexpert.rtd",,"14597","KBFA020")</f>
-        <v>16</v>
-      </c>
-      <c r="G11" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="G11" s="9"/>
       <c r="L11" s="4">
         <f>RTD("checkexpert.rtd",,"14535","KXFA020")</f>
-        <v>106.25</v>
+        <v>106.69</v>
       </c>
       <c r="M11" s="1">
         <f>RTD("checkexpert.rtd",,"14545","KXFA020")</f>
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="N11" s="1">
         <f>RTD("checkexpert.rtd",,"14597","KXFA020")</f>
-        <v>4</v>
-      </c>
-      <c r="O11" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="O11" s="9"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B12">
         <f>RTD("checkexpert.rtd",,"14625","KBFA020")</f>
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="C12">
         <f>RTD("checkexpert.rtd",,"14621","KBFA020")</f>
-        <v>2184</v>
+        <v>1705</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
         <f>RTD("checkexpert.rtd",,"14623","KBFA020")</f>
-        <v>3402</v>
+        <v>2062</v>
       </c>
       <c r="F12">
         <f>RTD("checkexpert.rtd",,"14627","KBFA020")</f>
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="J12">
         <f>RTD("checkexpert.rtd",,"14625","KXFA020")</f>
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="K12">
         <f>RTD("checkexpert.rtd",,"14621","KXFA020")</f>
-        <v>380</v>
+        <v>500</v>
       </c>
       <c r="M12">
         <f>RTD("checkexpert.rtd",,"14623","KXFA020")</f>
-        <v>501</v>
+        <v>474</v>
       </c>
       <c r="N12">
         <f>RTD("checkexpert.rtd",,"14627","KXFA020")</f>
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -1515,7 +1526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.25" bestFit="1" customWidth="1"/>
@@ -1528,7 +1539,7 @@
       </c>
       <c r="B1">
         <f>RTD("checkexpert.rtd",,"15175","KTBS03*161")</f>
-        <v>3.8610000000000002</v>
+        <v>3.8220000000000001</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1537,25 +1548,25 @@
       </c>
       <c r="B2">
         <f>RTD("checkexpert.rtd",,"15175","KTBS10*161")</f>
-        <v>4.1879999999999997</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="7">
         <f>RTD("checkexpert.rtd",,"17967^11","*017")</f>
-        <v>119111</v>
+        <v>94277</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="7">
         <f>RTD("checkexpert.rtd",,"17966^11","*017")</f>
-        <v>118204</v>
+        <v>90642</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1564,7 +1575,7 @@
       </c>
       <c r="B5">
         <f>RTD("checkexpert.rtd",,"15001","KBFA020")</f>
-        <v>102.95</v>
+        <v>103.14</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -1573,25 +1584,25 @@
       </c>
       <c r="B6">
         <f>RTD("checkexpert.rtd",,"15175","KBFA020")</f>
-        <v>3.948</v>
+        <v>3.8809999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="7">
         <f>RTD("checkexpert.rtd",,"17967^11","*016")</f>
-        <v>78687</v>
+        <v>53035</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="7">
         <f>RTD("checkexpert.rtd",,"17966^11","*016")</f>
-        <v>78086</v>
+        <v>52663</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -1600,7 +1611,7 @@
       </c>
       <c r="B9">
         <f>RTD("checkexpert.rtd",,"15001","KXFA020")</f>
-        <v>106.3</v>
+        <v>106.76</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -1609,7 +1620,16 @@
       </c>
       <c r="B10">
         <f>RTD("checkexpert.rtd",,"15175","KXFA020")</f>
-        <v>4.2210000000000001</v>
+        <v>4.1669999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11">
+        <f>RTD("checkexpert.rtd",,"15175","KTBS05*161")</f>
+        <v>3.9649999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>